<commit_message>
Patrimoniale importer as rest api
</commit_message>
<xml_diff>
--- a/PatrimonialeImporter/PatrimonialeImporter/Resources/PatrimonialeData.xlsx
+++ b/PatrimonialeImporter/PatrimonialeImporter/Resources/PatrimonialeData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\addressfeapp\PatrimonialeImporter\PatrimonialeImporter\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6F35E47-3AC9-4581-8309-5DCEBAE3FB8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4BB5D87-72A9-41F3-81F8-E0E183256230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1680" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
   <si>
     <t>employmentStatus</t>
   </si>
@@ -100,15 +100,6 @@
   </si>
   <si>
     <t>SelfEmployed</t>
-  </si>
-  <si>
-    <t>client</t>
-  </si>
-  <si>
-    <t>clientId</t>
-  </si>
-  <si>
-    <t>019fa850-d8fb-75a3-ac19-39c8ef1e2e5f</t>
   </si>
   <si>
     <t>Permament</t>
@@ -177,13 +168,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -470,10 +458,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O4"/>
+  <dimension ref="B1:O4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -489,37 +476,31 @@
     <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="5" t="s">
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="5"/>
-      <c r="J1" s="4" t="s">
+      <c r="I1" s="4"/>
+      <c r="J1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="5" t="s">
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>26</v>
-      </c>
+    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -563,10 +544,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>27</v>
-      </c>
+    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>18</v>
       </c>
@@ -574,7 +552,7 @@
         <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
         <v>20</v>
@@ -601,10 +579,7 @@
         <v>46054</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>27</v>
-      </c>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>24</v>
       </c>

</xml_diff>

<commit_message>
Reading excel from directory
</commit_message>
<xml_diff>
--- a/PatrimonialeImporter/PatrimonialeImporter/Resources/PatrimonialeData.xlsx
+++ b/PatrimonialeImporter/PatrimonialeImporter/Resources/PatrimonialeData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\addressfeapp\PatrimonialeImporter\PatrimonialeImporter\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4BB5D87-72A9-41F3-81F8-E0E183256230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE4301F-884E-4DAF-A7D7-32CD72E57A4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1680" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>

</xml_diff>